<commit_message>
Add FedTSPv2. Plave the textencoder on the server.
</commit_message>
<xml_diff>
--- a/实验记录.xlsx
+++ b/实验记录.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ResearchCode\Idea\HtFLlib-1.8.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuxinghao/Documents/联邦学习/ResearchCode/FedTSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0640F0EC-7CD9-47D7-9905-5964368903C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4DE11B-160B-FD4A-A33E-B7BD4B2869EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21390" yWindow="4815" windowWidth="20475" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28620" yWindow="-8380" windowWidth="28600" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="30">
   <si>
     <t>验证文本prompt对训练的影响</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -149,6 +149,10 @@
   </si>
   <si>
     <t>alter 4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>18.58 on 3090, p_prompt=1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -156,7 +160,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -474,15 +478,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q60"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:S60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -502,7 +506,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -513,7 +517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -527,7 +531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>1</v>
       </c>
@@ -544,7 +548,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>1</v>
       </c>
@@ -561,7 +565,7 @@
         <v>84.57</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>0</v>
       </c>
@@ -581,7 +585,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -601,7 +605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -609,7 +613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -623,7 +627,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>1</v>
       </c>
@@ -637,7 +641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>1</v>
       </c>
@@ -657,7 +661,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>0</v>
       </c>
@@ -677,7 +681,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>2</v>
       </c>
@@ -694,7 +698,7 @@
         <v>53.74</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>3</v>
       </c>
@@ -714,7 +718,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>2</v>
       </c>
@@ -725,7 +729,7 @@
         <v>55.36</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>3</v>
       </c>
@@ -736,7 +740,7 @@
         <v>55.58</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>4</v>
       </c>
@@ -747,7 +751,7 @@
         <v>56.52</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>4</v>
       </c>
@@ -758,7 +762,7 @@
         <v>55.68</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>4</v>
       </c>
@@ -772,7 +776,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>10</v>
       </c>
@@ -783,7 +787,7 @@
         <v>56.19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>5</v>
       </c>
@@ -794,7 +798,7 @@
         <v>55.72</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>5</v>
       </c>
@@ -805,7 +809,7 @@
         <v>56.91</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>5</v>
       </c>
@@ -819,7 +823,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>6</v>
       </c>
@@ -830,7 +834,7 @@
         <v>56.93</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>6</v>
       </c>
@@ -844,7 +848,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>7</v>
       </c>
@@ -855,7 +859,7 @@
         <v>56.64</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>7</v>
       </c>
@@ -869,7 +873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>8</v>
       </c>
@@ -880,7 +884,7 @@
         <v>56.66</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>8</v>
       </c>
@@ -894,7 +898,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19">
       <c r="A33">
         <v>7</v>
       </c>
@@ -908,7 +912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19">
       <c r="A34">
         <v>7</v>
       </c>
@@ -919,7 +923,7 @@
         <v>56.66</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19">
       <c r="A35">
         <v>7</v>
       </c>
@@ -933,7 +937,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19">
       <c r="B37" t="s">
         <v>19</v>
       </c>
@@ -947,7 +951,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19">
       <c r="A38" t="s">
         <v>20</v>
       </c>
@@ -958,15 +962,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19">
       <c r="J39" t="s">
         <v>25</v>
       </c>
-      <c r="N39" t="s">
+      <c r="P39" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -991,20 +995,20 @@
       <c r="L40" t="s">
         <v>23</v>
       </c>
-      <c r="N40" t="s">
-        <v>1</v>
-      </c>
-      <c r="O40" t="s">
-        <v>6</v>
-      </c>
       <c r="P40" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>6</v>
+      </c>
+      <c r="R40" t="s">
         <v>27</v>
       </c>
-      <c r="Q40" t="s">
+      <c r="S40" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19">
       <c r="J41">
         <v>0</v>
       </c>
@@ -1014,14 +1018,14 @@
       <c r="L41">
         <v>300</v>
       </c>
-      <c r="N41">
-        <v>1</v>
-      </c>
-      <c r="O41">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P41">
+        <v>1</v>
+      </c>
+      <c r="Q41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19">
       <c r="J42">
         <v>1</v>
       </c>
@@ -1031,20 +1035,20 @@
       <c r="L42">
         <v>300</v>
       </c>
-      <c r="N42">
+      <c r="P42">
         <v>2</v>
       </c>
-      <c r="O42">
-        <v>5</v>
-      </c>
-      <c r="P42">
+      <c r="Q42">
+        <v>5</v>
+      </c>
+      <c r="R42">
         <v>17.38</v>
       </c>
-      <c r="Q42">
+      <c r="S42">
         <v>219</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19">
       <c r="J43">
         <v>2</v>
       </c>
@@ -1054,17 +1058,17 @@
       <c r="L43">
         <v>300</v>
       </c>
-      <c r="N43">
+      <c r="P43">
         <v>3</v>
       </c>
-      <c r="O43">
-        <v>5</v>
-      </c>
-      <c r="P43">
+      <c r="Q43">
+        <v>5</v>
+      </c>
+      <c r="R43">
         <v>17.82</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19">
       <c r="J44">
         <v>3</v>
       </c>
@@ -1074,17 +1078,17 @@
       <c r="L44">
         <v>300</v>
       </c>
-      <c r="N44">
+      <c r="P44">
         <v>4</v>
       </c>
-      <c r="O44">
-        <v>5</v>
-      </c>
-      <c r="P44">
+      <c r="Q44">
+        <v>5</v>
+      </c>
+      <c r="R44">
         <v>18.04</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19">
       <c r="J45">
         <v>4</v>
       </c>
@@ -1094,17 +1098,17 @@
       <c r="L45">
         <v>300</v>
       </c>
-      <c r="N45">
-        <v>5</v>
-      </c>
-      <c r="O45">
-        <v>5</v>
-      </c>
       <c r="P45">
+        <v>5</v>
+      </c>
+      <c r="Q45">
+        <v>5</v>
+      </c>
+      <c r="R45">
         <v>18.09</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19">
       <c r="J46">
         <v>5</v>
       </c>
@@ -1114,17 +1118,17 @@
       <c r="L46">
         <v>300</v>
       </c>
-      <c r="N46">
-        <v>6</v>
-      </c>
-      <c r="O46">
-        <v>5</v>
-      </c>
       <c r="P46">
+        <v>6</v>
+      </c>
+      <c r="Q46">
+        <v>5</v>
+      </c>
+      <c r="R46">
         <v>18.14</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19">
       <c r="J47">
         <v>6</v>
       </c>
@@ -1134,17 +1138,20 @@
       <c r="L47">
         <v>300</v>
       </c>
-      <c r="N47">
+      <c r="M47" t="s">
+        <v>29</v>
+      </c>
+      <c r="P47">
         <v>7</v>
       </c>
-      <c r="O47">
-        <v>5</v>
-      </c>
-      <c r="P47">
+      <c r="Q47">
+        <v>5</v>
+      </c>
+      <c r="R47">
         <v>18.55</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19">
       <c r="J48">
         <v>7</v>
       </c>
@@ -1154,17 +1161,17 @@
       <c r="L48">
         <v>100</v>
       </c>
-      <c r="N48">
+      <c r="P48">
         <v>8</v>
       </c>
-      <c r="O48">
-        <v>5</v>
-      </c>
-      <c r="P48">
+      <c r="Q48">
+        <v>5</v>
+      </c>
+      <c r="R48">
         <v>18.260000000000002</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19">
       <c r="A49">
         <v>6</v>
       </c>
@@ -1190,7 +1197,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19">
       <c r="A50">
         <v>6</v>
       </c>
@@ -1207,7 +1214,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19">
       <c r="A51">
         <v>6</v>
       </c>
@@ -1229,11 +1236,11 @@
       <c r="J51" t="s">
         <v>17</v>
       </c>
-      <c r="N51" t="s">
+      <c r="P51" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19">
       <c r="J52" t="s">
         <v>1</v>
       </c>
@@ -1243,76 +1250,76 @@
       <c r="L52" t="s">
         <v>27</v>
       </c>
-      <c r="N52" t="s">
-        <v>1</v>
-      </c>
-      <c r="O52" t="s">
-        <v>6</v>
-      </c>
       <c r="P52" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>6</v>
+      </c>
+      <c r="R52" t="s">
         <v>27</v>
       </c>
-      <c r="Q52" t="s">
+      <c r="S52" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19">
       <c r="J53">
         <v>1</v>
       </c>
       <c r="K53">
         <v>5</v>
       </c>
-      <c r="N53">
-        <v>1</v>
-      </c>
-      <c r="O53">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P53">
+        <v>1</v>
+      </c>
+      <c r="Q53">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19">
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54">
         <v>5</v>
       </c>
-      <c r="N54">
+      <c r="P54">
         <v>2</v>
       </c>
-      <c r="O54">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="Q54">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19">
       <c r="J55">
         <v>3</v>
       </c>
       <c r="K55">
         <v>5</v>
       </c>
-      <c r="N55">
+      <c r="P55">
         <v>3</v>
       </c>
-      <c r="O55">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="Q55">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19">
       <c r="J56">
         <v>4</v>
       </c>
       <c r="K56">
         <v>5</v>
       </c>
-      <c r="N56">
+      <c r="P56">
         <v>4</v>
       </c>
-      <c r="O56">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="Q56">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19">
       <c r="J57">
         <v>5</v>
       </c>
@@ -1322,17 +1329,17 @@
       <c r="L57">
         <v>18.45</v>
       </c>
-      <c r="N57">
-        <v>5</v>
-      </c>
-      <c r="O57">
-        <v>5</v>
-      </c>
       <c r="P57">
+        <v>5</v>
+      </c>
+      <c r="Q57">
+        <v>5</v>
+      </c>
+      <c r="R57">
         <v>18.34</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19">
       <c r="J58">
         <v>6</v>
       </c>
@@ -1342,44 +1349,44 @@
       <c r="L58">
         <v>18.91</v>
       </c>
-      <c r="N58">
-        <v>6</v>
-      </c>
-      <c r="O58">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P58">
+        <v>6</v>
+      </c>
+      <c r="Q58">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19">
       <c r="J59">
         <v>7</v>
       </c>
       <c r="K59">
         <v>5</v>
       </c>
-      <c r="N59">
+      <c r="P59">
         <v>7</v>
       </c>
-      <c r="O59">
-        <v>5</v>
-      </c>
-      <c r="P59">
+      <c r="Q59">
+        <v>5</v>
+      </c>
+      <c r="R59">
         <v>19.010000000000002</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19">
       <c r="J60">
         <v>8</v>
       </c>
       <c r="K60">
         <v>5</v>
       </c>
-      <c r="N60">
+      <c r="P60">
         <v>8</v>
       </c>
-      <c r="O60">
-        <v>5</v>
-      </c>
-      <c r="P60">
+      <c r="Q60">
+        <v>5</v>
+      </c>
+      <c r="R60">
         <v>18.63</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FedTSPv3: 1) allow to use bert as the global text encoder; 2) logit_scale is trainable and shared by server.
</commit_message>
<xml_diff>
--- a/实验记录.xlsx
+++ b/实验记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuxinghao/Documents/联邦学习/ResearchCode/FedTSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D776B910-A0FA-5841-87A6-5DA13CB2A55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF4E6CF-9E4D-6C40-90FD-29CBD52009BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28880" yWindow="-24340" windowWidth="28620" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CIFAR100-dir1.0-client20" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="61">
   <si>
     <t>验证文本prompt对训练的影响</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -277,6 +277,10 @@
   </si>
   <si>
     <t>update</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>500 rounds</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -623,10 +627,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CCDCA62-1458-6748-AAD6-300D2625CB6F}">
-  <dimension ref="A1:Q118"/>
+  <dimension ref="A1:S118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:19">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -643,7 +647,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -680,11 +684,17 @@
       <c r="M2" t="s">
         <v>10</v>
       </c>
-      <c r="P2" t="s">
+      <c r="N2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>1</v>
       </c>
@@ -721,14 +731,20 @@
       <c r="N3" t="s">
         <v>27</v>
       </c>
-      <c r="P3" t="s">
-        <v>1</v>
+      <c r="O3" t="s">
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:17">
+      <c r="S3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>2</v>
       </c>
@@ -765,14 +781,14 @@
       <c r="N4">
         <v>15.99</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>0.1</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>20.25</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>3</v>
       </c>
@@ -806,11 +822,23 @@
       <c r="M5">
         <v>0.2</v>
       </c>
-      <c r="P5">
+      <c r="N5">
+        <v>17.12</v>
+      </c>
+      <c r="O5">
+        <v>495</v>
+      </c>
+      <c r="Q5">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:17">
+      <c r="R5">
+        <v>20.329999999999998</v>
+      </c>
+      <c r="S5">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>4</v>
       </c>
@@ -844,11 +872,23 @@
       <c r="M6">
         <v>0.3</v>
       </c>
-      <c r="P6">
+      <c r="N6">
+        <v>17.38</v>
+      </c>
+      <c r="O6">
+        <v>237</v>
+      </c>
+      <c r="Q6">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="7" spans="1:17">
+      <c r="R6">
+        <v>20.6</v>
+      </c>
+      <c r="S6">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>5</v>
       </c>
@@ -882,11 +922,23 @@
       <c r="M7">
         <v>0.4</v>
       </c>
-      <c r="P7">
+      <c r="N7">
+        <v>17.809999999999999</v>
+      </c>
+      <c r="O7">
+        <v>471</v>
+      </c>
+      <c r="Q7">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="8" spans="1:17">
+      <c r="R7">
+        <v>20.98</v>
+      </c>
+      <c r="S7">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>6</v>
       </c>
@@ -920,11 +972,23 @@
       <c r="M8">
         <v>0.5</v>
       </c>
-      <c r="P8">
+      <c r="N8">
+        <v>18.079999999999998</v>
+      </c>
+      <c r="O8">
+        <v>370</v>
+      </c>
+      <c r="Q8">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:17">
+      <c r="R8">
+        <v>20.89</v>
+      </c>
+      <c r="S8">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>7</v>
       </c>
@@ -956,7 +1020,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>8</v>
       </c>
@@ -988,7 +1052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1017,17 +1081,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:19">
       <c r="A12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:19">
       <c r="A13">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:19">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -1062,7 +1126,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:19">
       <c r="A16">
         <v>1</v>
       </c>
@@ -3629,10 +3693,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFB62DF-B5AA-5E4C-80E6-11565E9C9DBC}">
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:19">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -3649,7 +3713,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -3686,11 +3750,17 @@
       <c r="M2" t="s">
         <v>10</v>
       </c>
-      <c r="P2" t="s">
+      <c r="N2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3727,14 +3797,20 @@
       <c r="N3" t="s">
         <v>27</v>
       </c>
-      <c r="P3" t="s">
-        <v>1</v>
+      <c r="O3" t="s">
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:17">
+      <c r="S3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3771,14 +3847,14 @@
       <c r="N4">
         <v>56.39</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>0.1</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>58.37</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3815,14 +3891,14 @@
       <c r="N5">
         <v>56.94</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>0.2</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>58.81</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3859,14 +3935,14 @@
       <c r="N6">
         <v>57.27</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>0.3</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>58.84</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3900,11 +3976,23 @@
       <c r="M7">
         <v>0.4</v>
       </c>
-      <c r="P7">
+      <c r="N7">
+        <v>57.1</v>
+      </c>
+      <c r="O7">
+        <v>422</v>
+      </c>
+      <c r="Q7">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="8" spans="1:17">
+      <c r="R7">
+        <v>59.13</v>
+      </c>
+      <c r="S7">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3938,11 +4026,23 @@
       <c r="M8">
         <v>0.5</v>
       </c>
-      <c r="P8">
+      <c r="N8">
+        <v>57.15</v>
+      </c>
+      <c r="O8">
+        <v>423</v>
+      </c>
+      <c r="Q8">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:17">
+      <c r="R8">
+        <v>58.89</v>
+      </c>
+      <c r="S8">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3974,7 +4074,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4006,22 +4106,22 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:19">
       <c r="A12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:19">
       <c r="A13">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:19">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -4056,7 +4156,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:19">
       <c r="A16">
         <v>1</v>
       </c>

</xml_diff>